<commit_message>
feat(corpus): revamp PedalWorks kb-test into a 3-tier hierarchical corpus
Rewrites the synthetic PedalWorks corpus so extraction yields a clean, tiered knowledge graph (Tier 0 super-themes -> Tier 1 sub-nodes -> Tier 2 detail):
- item-first supplier names (Frames Ltd, Wheels Co, ...); dropped generic 'Bicycle'; Scheduler -> Planner
- new docs: architecture-flow, data-model, bom, production, fulfillment, planning_and_demand
- prose<->code twin kept; binaries regenerated with image/table probes preserved
- dropped Dockerfile/Makefile (were ingested as infra noise)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/inventory_stock.xlsx
+++ b/data/inventory_stock.xlsx
@@ -413,36 +413,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Stock Record</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Lead Time</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Qty On Hand</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Reorder Threshold</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Safety Stock</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Unit Cost</t>
         </is>
@@ -451,130 +461,170 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Frame Stock</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Frame</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>FrameForge Ltd</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North Intake Warehouse</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>340</v>
+          <t>Frames Ltd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>14 days</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
         <v>120</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Wheelset Stock</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Wheelset</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RollRight Co</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North Intake Warehouse</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>512</v>
+          <t>Wheels Co</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>150</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
         <v>85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Drivetrain Stock</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Drivetrain</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GearWorks Inc</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>North Intake Warehouse</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>208</v>
+          <t>Drivetrain Co</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10 days</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
         <v>95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Brake Set Stock</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Brake Set</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BrakeSafe GmbH</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>North Intake Warehouse</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>275</v>
+          <t>Brakes Ltd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>10 days</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Suspension Fork Stock</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Suspension Fork</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ForkFactory Co</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North Intake Warehouse</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>64</v>
+          <t>Forks Co</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12 days</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
         <v>150</v>
       </c>
     </row>

</xml_diff>